<commit_message>
Update ELC and SUP for URAN IMPORT
</commit_message>
<xml_diff>
--- a/VT_Model_SUP_V01.xlsx
+++ b/VT_Model_SUP_V01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr showObjects="placeholders" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\bbb\MSc_SELECT-main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yukiainge/Downloads/UPC - Energy Modeling &amp; Climate Policy/TIMES/MSc_SELECT-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3B79E5-BAF8-41F8-8ADC-A66F838D3F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23A179B3-979D-3442-830A-6CDF7D130999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="901" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15840" tabRatio="901" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEC_Comm" sheetId="112" r:id="rId1"/>
@@ -784,7 +784,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="101">
   <si>
     <t>Define Commodities</t>
   </si>
@@ -1075,6 +1075,18 @@
   </si>
   <si>
     <t>ANNUAL</t>
+  </si>
+  <si>
+    <t>URAN</t>
+  </si>
+  <si>
+    <t>Uranium Fuel</t>
+  </si>
+  <si>
+    <t>PF</t>
+  </si>
+  <si>
+    <t>IMP_URAN</t>
   </si>
 </sst>
 </file>
@@ -2587,6 +2599,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="IEA Data"/>
       <sheetName val="E&amp;D Drivers"/>
@@ -3069,18 +3084,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="B2:I29"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" customWidth="1"/>
-    <col min="2" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="10" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="10" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="18">
@@ -3115,7 +3130,7 @@
       <c r="H4" s="26"/>
       <c r="I4" s="26"/>
     </row>
-    <row r="5" spans="2:9">
+    <row r="5" spans="2:9" ht="14">
       <c r="B5" s="27" t="s">
         <v>2</v>
       </c>
@@ -3141,7 +3156,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="38.25">
+    <row r="6" spans="2:9" ht="28">
       <c r="B6" s="37" t="s">
         <v>10</v>
       </c>
@@ -3270,10 +3285,22 @@
       </c>
     </row>
     <row r="12" spans="2:9">
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="E12" s="23"/>
+      <c r="B12" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>99</v>
+      </c>
       <c r="F12" s="18"/>
+      <c r="G12" s="20" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="13" spans="2:9">
       <c r="F13" s="18"/>
@@ -3321,7 +3348,7 @@
       <c r="C22" s="23"/>
       <c r="E22" s="23"/>
     </row>
-    <row r="24" spans="2:5" ht="13.5" thickBot="1">
+    <row r="24" spans="2:5" ht="14" thickBot="1">
       <c r="B24" s="38" t="s">
         <v>18</v>
       </c>
@@ -3359,7 +3386,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="2:5" ht="13.5" thickBot="1">
+    <row r="29" spans="2:5" ht="14" thickBot="1">
       <c r="B29" s="22" t="s">
         <v>26</v>
       </c>
@@ -3382,18 +3409,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:J31"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="28.5703125" customWidth="1"/>
+    <col min="5" max="5" width="28.5" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="11.5" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="13" max="13" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="18" customHeight="1">
@@ -3581,6 +3608,23 @@
       <c r="I11" s="21"/>
       <c r="J11" s="21"/>
     </row>
+    <row r="12" spans="1:10">
+      <c r="B12" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>96</v>
+      </c>
+    </row>
     <row r="15" spans="1:10">
       <c r="B15" s="23"/>
       <c r="C15" s="23"/>
@@ -3697,7 +3741,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="2:6" ht="13.5" thickBot="1">
+    <row r="31" spans="2:6" ht="14" thickBot="1">
       <c r="B31" s="22" t="s">
         <v>66</v>
       </c>
@@ -3721,14 +3765,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:T26"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="27.28515625" customWidth="1"/>
-    <col min="4" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="10" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" customWidth="1"/>
+    <col min="4" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="10" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -3966,6 +4010,16 @@
       <c r="J11" s="5"/>
     </row>
     <row r="12" spans="1:20">
+      <c r="B12" t="str">
+        <f>SEC_Processes!D12</f>
+        <v>IMP_URAN</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E12">
+        <v>0.5</v>
+      </c>
       <c r="F12" s="5"/>
       <c r="H12" s="14"/>
       <c r="I12" s="5"/>
@@ -4054,21 +4108,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E800C01780957C4993EAD0B0EDC5E8FF" ma:contentTypeVersion="4" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="56d16bfd38a93d3246b87ec2f908dfef">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="95645557-b925-4e14-b9c3-bb0dccab904e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e7776de10091f04de0bec4c5ba2ee03" ns2:_="">
     <xsd:import namespace="95645557-b925-4e14-b9c3-bb0dccab904e"/>
@@ -4212,24 +4251,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2354E624-82C6-4C58-B5AA-5F4B4FEE1585}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BEC55BD-C1AB-47C6-923C-1E0B74C138B9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4ADE2FD8-87C7-41E1-A1A0-6DF35B741F42}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4245,4 +4282,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BEC55BD-C1AB-47C6-923C-1E0B74C138B9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2354E624-82C6-4C58-B5AA-5F4B4FEE1585}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>